<commit_message>
Fix hedging-set row references in IR aggregation (C42, C43)
</commit_message>
<xml_diff>
--- a/SA-CCR Model.xlsx
+++ b/SA-CCR Model.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Desktop\My website\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70680CBF-1923-4765-A061-3DF5501568E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B285F07A-F0A6-4C5D-8C68-EA506357D9C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{292C9C36-5BD6-4200-9D09-254E443E619D}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{292C9C36-5BD6-4200-9D09-254E443E619D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
     <definedName name="count">#REF!</definedName>
     <definedName name="worth">#REF!</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -2798,7 +2798,7 @@
         <v>41</v>
       </c>
       <c r="C42" s="4">
-        <f t="shared" ref="C42:C43" si="2" xml:space="preserve"> SUMIFS($AD$23:$AD$34,$D$23:$D$34,B43,$AE$23:$AE$34,1)</f>
+        <f t="shared" ref="C42:C43" si="2" xml:space="preserve"> SUMIFS($AD$23:$AD$34,$D$23:$D$34,B42,$AE$23:$AE$34,1)</f>
         <v>0</v>
       </c>
       <c r="D42" s="4">

</xml_diff>